<commit_message>
Add parameter for Kg/pallet sensitivity analysis
</commit_message>
<xml_diff>
--- a/in/gaza_food_data.xlsx
+++ b/in/gaza_food_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\mortality_estimation_crises\gaza 2023-2024\gaza_nutrition_papers\caloric_availability\revised\in\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\mortality_estimation_crises\gaza_2023-2024\gaza_nutrition_papers\caloric_availability\revised\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{336E4A03-52A1-48FA-B326-C3F80734894A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87AF4B71-29BA-4E4F-9ADA-AD930087CEAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="14" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1754" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="481">
   <si>
     <t>North Gaza</t>
   </si>
@@ -1490,6 +1490,15 @@
   </si>
   <si>
     <t>sensitivity?</t>
+  </si>
+  <si>
+    <t>pallet_bias</t>
+  </si>
+  <si>
+    <t>systematic bias in assumed pallet weight</t>
+  </si>
+  <si>
+    <t>relative; 0 assumed for main analysis; sensitivity analysis: +0.2 to -0.2</t>
   </si>
 </sst>
 </file>
@@ -2174,7 +2183,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" style="35" bestFit="1" customWidth="1"/>
@@ -2290,45 +2299,59 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="27" x14ac:dyDescent="0.25">
       <c r="A9" s="35" t="s">
-        <v>144</v>
+        <v>478</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>145</v>
+        <v>479</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>146</v>
+        <v>480</v>
       </c>
       <c r="D9" s="35">
-        <v>5.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="35" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>420</v>
+        <v>145</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>1</v>
-      </c>
-      <c r="D10" s="41">
-        <v>38349604452</v>
+        <v>146</v>
+      </c>
+      <c r="D10" s="35">
+        <v>5.6</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" s="40" t="s">
+        <v>420</v>
+      </c>
+      <c r="C11" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="41">
+        <v>38349604452</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B12" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="C11" s="40" t="s">
+      <c r="C12" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="42" t="s">
+      <c r="D12" s="42" t="s">
         <v>150</v>
       </c>
     </row>

</xml_diff>